<commit_message>
fix: import students file 2.0
</commit_message>
<xml_diff>
--- a/attendance-frontend/admin/assets/documents/student_import_template.xlsx
+++ b/attendance-frontend/admin/assets/documents/student_import_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -419,9 +419,29 @@
         <v>phone_number</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>SV01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Nguyen Van A</v>
+      </c>
+      <c r="C2" t="str">
+        <v>nva@email.com</v>
+      </c>
+      <c r="D2" t="str">
+        <v>64HTTT1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Nam</v>
+      </c>
+      <c r="F2" t="str">
+        <v>0123456789</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>